<commit_message>
correzione laminati iniziali non 12 ma 9
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto/FOLDER/EXCEL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBCA013-7BF3-45EC-924C-2A95B24A8595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCED0509-6097-402A-8FBE-051F34920DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="68">
   <si>
     <t>Petri net incidence and marking</t>
   </si>
@@ -291,6 +291,21 @@
   <si>
     <t>descrizione</t>
   </si>
+  <si>
+    <t xml:space="preserve"> 1/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/6</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/5</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/3</t>
+  </si>
 </sst>
 </file>
 
@@ -433,10 +448,10 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -728,26 +743,26 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
+      <c r="A3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
     </row>
     <row r="4" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -2428,26 +2443,26 @@
       </c>
     </row>
     <row r="34" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
-      <c r="Q34" s="8"/>
-      <c r="R34" s="8"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
+      <c r="N34" s="7"/>
+      <c r="O34" s="7"/>
+      <c r="P34" s="7"/>
+      <c r="Q34" s="7"/>
+      <c r="R34" s="7"/>
     </row>
     <row r="35" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -4128,26 +4143,26 @@
       </c>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A65" s="8" t="s">
+      <c r="A65" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B65" s="8"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="8"/>
-      <c r="E65" s="8"/>
-      <c r="F65" s="8"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="8"/>
-      <c r="I65" s="8"/>
-      <c r="J65" s="8"/>
-      <c r="K65" s="8"/>
-      <c r="L65" s="8"/>
-      <c r="M65" s="8"/>
-      <c r="N65" s="8"/>
-      <c r="O65" s="8"/>
-      <c r="P65" s="8"/>
-      <c r="Q65" s="8"/>
-      <c r="R65" s="8"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="7"/>
+      <c r="I65" s="7"/>
+      <c r="J65" s="7"/>
+      <c r="K65" s="7"/>
+      <c r="L65" s="7"/>
+      <c r="M65" s="7"/>
+      <c r="N65" s="7"/>
+      <c r="O65" s="7"/>
+      <c r="P65" s="7"/>
+      <c r="Q65" s="7"/>
+      <c r="R65" s="7"/>
     </row>
     <row r="66" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
@@ -5828,26 +5843,26 @@
       </c>
     </row>
     <row r="96" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A96" s="8" t="s">
+      <c r="A96" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B96" s="8"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="8"/>
-      <c r="E96" s="8"/>
-      <c r="F96" s="8"/>
-      <c r="G96" s="8"/>
-      <c r="H96" s="8"/>
-      <c r="I96" s="8"/>
-      <c r="J96" s="8"/>
-      <c r="K96" s="8"/>
-      <c r="L96" s="8"/>
-      <c r="M96" s="8"/>
-      <c r="N96" s="8"/>
-      <c r="O96" s="8"/>
-      <c r="P96" s="8"/>
-      <c r="Q96" s="8"/>
-      <c r="R96" s="8"/>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="7"/>
+      <c r="E96" s="7"/>
+      <c r="F96" s="7"/>
+      <c r="G96" s="7"/>
+      <c r="H96" s="7"/>
+      <c r="I96" s="7"/>
+      <c r="J96" s="7"/>
+      <c r="K96" s="7"/>
+      <c r="L96" s="7"/>
+      <c r="M96" s="7"/>
+      <c r="N96" s="7"/>
+      <c r="O96" s="7"/>
+      <c r="P96" s="7"/>
+      <c r="Q96" s="7"/>
+      <c r="R96" s="7"/>
     </row>
     <row r="97" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
@@ -7528,38 +7543,38 @@
       </c>
     </row>
     <row r="127" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A127" s="8" t="s">
+      <c r="A127" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B127" s="8"/>
-      <c r="C127" s="8"/>
-      <c r="D127" s="8"/>
-      <c r="E127" s="8"/>
-      <c r="F127" s="8"/>
-      <c r="G127" s="8"/>
-      <c r="H127" s="8"/>
-      <c r="I127" s="8"/>
-      <c r="J127" s="8"/>
-      <c r="K127" s="8"/>
-      <c r="L127" s="8"/>
-      <c r="M127" s="8"/>
-      <c r="N127" s="8"/>
-      <c r="O127" s="8"/>
-      <c r="P127" s="8"/>
-      <c r="Q127" s="8"/>
-      <c r="R127" s="8"/>
-      <c r="S127" s="8"/>
-      <c r="T127" s="8"/>
-      <c r="U127" s="8"/>
-      <c r="V127" s="8"/>
-      <c r="W127" s="8"/>
-      <c r="X127" s="8"/>
-      <c r="Y127" s="8"/>
-      <c r="Z127" s="8"/>
-      <c r="AA127" s="8"/>
-      <c r="AB127" s="8"/>
-      <c r="AC127" s="8"/>
-      <c r="AD127" s="8"/>
+      <c r="B127" s="7"/>
+      <c r="C127" s="7"/>
+      <c r="D127" s="7"/>
+      <c r="E127" s="7"/>
+      <c r="F127" s="7"/>
+      <c r="G127" s="7"/>
+      <c r="H127" s="7"/>
+      <c r="I127" s="7"/>
+      <c r="J127" s="7"/>
+      <c r="K127" s="7"/>
+      <c r="L127" s="7"/>
+      <c r="M127" s="7"/>
+      <c r="N127" s="7"/>
+      <c r="O127" s="7"/>
+      <c r="P127" s="7"/>
+      <c r="Q127" s="7"/>
+      <c r="R127" s="7"/>
+      <c r="S127" s="7"/>
+      <c r="T127" s="7"/>
+      <c r="U127" s="7"/>
+      <c r="V127" s="7"/>
+      <c r="W127" s="7"/>
+      <c r="X127" s="7"/>
+      <c r="Y127" s="7"/>
+      <c r="Z127" s="7"/>
+      <c r="AA127" s="7"/>
+      <c r="AB127" s="7"/>
+      <c r="AC127" s="7"/>
+      <c r="AD127" s="7"/>
     </row>
     <row r="128" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A128" s="2"/>
@@ -7659,7 +7674,7 @@
         <v>0</v>
       </c>
       <c r="C129" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D129" s="5">
         <v>1</v>
@@ -7686,7 +7701,7 @@
         <v>0</v>
       </c>
       <c r="L129" s="5">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="M129" s="5">
         <v>0</v>
@@ -7698,7 +7713,7 @@
         <v>0</v>
       </c>
       <c r="P129" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q129" s="5">
         <v>1</v>
@@ -7722,7 +7737,7 @@
         <v>0</v>
       </c>
       <c r="X129" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y129" s="5">
         <v>1</v>
@@ -7778,7 +7793,7 @@
         <v>0</v>
       </c>
       <c r="L130" s="6">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="M130" s="6">
         <v>0</v>
@@ -7836,25 +7851,25 @@
       </c>
     </row>
     <row r="131" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A131" s="8" t="s">
+      <c r="A131" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B131" s="8"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="8"/>
-      <c r="E131" s="8"/>
-      <c r="F131" s="8"/>
-      <c r="G131" s="8"/>
-      <c r="H131" s="8"/>
-      <c r="I131" s="8"/>
-      <c r="J131" s="8"/>
-      <c r="K131" s="8"/>
-      <c r="L131" s="8"/>
-      <c r="M131" s="8"/>
-      <c r="N131" s="8"/>
-      <c r="O131" s="8"/>
-      <c r="P131" s="8"/>
-      <c r="Q131" s="8"/>
+      <c r="B131" s="7"/>
+      <c r="C131" s="7"/>
+      <c r="D131" s="7"/>
+      <c r="E131" s="7"/>
+      <c r="F131" s="7"/>
+      <c r="G131" s="7"/>
+      <c r="H131" s="7"/>
+      <c r="I131" s="7"/>
+      <c r="J131" s="7"/>
+      <c r="K131" s="7"/>
+      <c r="L131" s="7"/>
+      <c r="M131" s="7"/>
+      <c r="N131" s="7"/>
+      <c r="O131" s="7"/>
+      <c r="P131" s="7"/>
+      <c r="Q131" s="7"/>
     </row>
     <row r="132" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
@@ -7967,56 +7982,56 @@
         <v>54</v>
       </c>
     </row>
-    <row r="135" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A135" t="s">
+    <row r="135" spans="1:30" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C135" t="s">
+      <c r="C135" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D135" t="s">
+      <c r="D135" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E135" t="s">
+      <c r="E135" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F135" t="s">
+      <c r="F135" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G135" t="s">
+      <c r="G135" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H135" t="s">
+      <c r="H135" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I135" t="s">
+      <c r="I135" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J135" t="s">
+      <c r="J135" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K135" t="s">
+      <c r="K135" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L135" t="s">
+      <c r="L135" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M135" t="s">
+      <c r="M135" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N135" t="s">
+      <c r="N135" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="O135" t="s">
+      <c r="O135" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="P135" t="s">
+      <c r="P135" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="Q135" t="s">
+      <c r="Q135" s="3" t="s">
         <v>18</v>
       </c>
     </row>
@@ -8137,14 +8152,14 @@
       </c>
     </row>
     <row r="140" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A140">
-        <v>2</v>
-      </c>
-      <c r="B140">
-        <v>6</v>
-      </c>
-      <c r="C140">
-        <v>2</v>
+      <c r="A140" t="s">
+        <v>63</v>
+      </c>
+      <c r="B140" t="s">
+        <v>64</v>
+      </c>
+      <c r="C140" t="s">
+        <v>63</v>
       </c>
       <c r="D140">
         <v>0</v>
@@ -8158,35 +8173,35 @@
       <c r="G140">
         <v>0</v>
       </c>
-      <c r="H140">
-        <v>2</v>
-      </c>
-      <c r="I140">
-        <v>5</v>
-      </c>
-      <c r="J140">
-        <v>2</v>
+      <c r="H140" t="s">
+        <v>63</v>
+      </c>
+      <c r="I140" t="s">
+        <v>65</v>
+      </c>
+      <c r="J140" t="s">
+        <v>63</v>
       </c>
       <c r="K140">
         <v>0</v>
       </c>
-      <c r="L140">
-        <v>2</v>
-      </c>
-      <c r="M140">
-        <v>5</v>
-      </c>
-      <c r="N140">
-        <v>2</v>
+      <c r="L140" t="s">
+        <v>63</v>
+      </c>
+      <c r="M140" t="s">
+        <v>65</v>
+      </c>
+      <c r="N140" t="s">
+        <v>63</v>
       </c>
       <c r="O140">
         <v>0</v>
       </c>
-      <c r="P140">
-        <v>8</v>
-      </c>
-      <c r="Q140">
-        <v>3</v>
+      <c r="P140" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q140" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="141" spans="1:30" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
aggiunta pezzo di codice nel main che non stampa il numero ma il nome del posto, inoltre aggiornati i vari file di indici di prestazione
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto/FOLDER/EXCEL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCED0509-6097-402A-8FBE-051F34920DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A83424-853D-49F7-9BB5-36E57C763FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="63">
   <si>
     <t>Petri net incidence and marking</t>
   </si>
@@ -291,21 +291,6 @@
   <si>
     <t>descrizione</t>
   </si>
-  <si>
-    <t xml:space="preserve"> 1/2</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/6</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/8</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/3</t>
-  </si>
 </sst>
 </file>
 
@@ -428,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -454,6 +439,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -8152,56 +8138,56 @@
       </c>
     </row>
     <row r="140" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
-        <v>63</v>
-      </c>
-      <c r="B140" t="s">
-        <v>64</v>
-      </c>
-      <c r="C140" t="s">
-        <v>63</v>
-      </c>
-      <c r="D140">
-        <v>0</v>
-      </c>
-      <c r="E140">
-        <v>0</v>
-      </c>
-      <c r="F140">
-        <v>0</v>
-      </c>
-      <c r="G140">
-        <v>0</v>
-      </c>
-      <c r="H140" t="s">
-        <v>63</v>
-      </c>
-      <c r="I140" t="s">
-        <v>65</v>
-      </c>
-      <c r="J140" t="s">
-        <v>63</v>
-      </c>
-      <c r="K140">
-        <v>0</v>
-      </c>
-      <c r="L140" t="s">
-        <v>63</v>
-      </c>
-      <c r="M140" t="s">
-        <v>65</v>
-      </c>
-      <c r="N140" t="s">
-        <v>63</v>
-      </c>
-      <c r="O140">
-        <v>0</v>
-      </c>
-      <c r="P140" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q140" t="s">
-        <v>67</v>
+      <c r="A140" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="B140" s="9">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="C140" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="D140" s="9">
+        <v>0</v>
+      </c>
+      <c r="E140" s="9">
+        <v>0</v>
+      </c>
+      <c r="F140" s="9">
+        <v>0</v>
+      </c>
+      <c r="G140" s="9">
+        <v>0</v>
+      </c>
+      <c r="H140" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="I140" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="J140" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="K140" s="9">
+        <v>0</v>
+      </c>
+      <c r="L140" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="M140" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="N140" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="O140" s="9">
+        <v>0</v>
+      </c>
+      <c r="P140" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="Q140" s="9">
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="141" spans="1:30" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update Excel e Matlab Buffer
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto/FOLDER/EXCEL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto\FOLDER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Buffer_Ridotto\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3612CE-D3FA-4FC9-9894-F9A4BBE3BF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBC5EA6-A548-4C1C-B546-765E68367DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5520" yWindow="3015" windowWidth="6330" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -721,14 +721,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AD147"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
@@ -750,7 +750,7 @@
       <c r="Q3" s="9"/>
       <c r="R3" s="9"/>
     </row>
-    <row r="4" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -804,7 +804,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
@@ -860,7 +860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
@@ -916,7 +916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
@@ -972,7 +972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>22</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>23</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>24</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>26</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>27</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>28</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>29</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>30</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>31</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>32</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>33</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>34</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>35</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>36</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>37</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>38</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>39</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>40</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>41</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>42</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>43</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>44</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>45</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>46</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>47</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>48</v>
       </c>
@@ -2450,7 +2450,7 @@
       <c r="Q34" s="8"/>
       <c r="R34" s="8"/>
     </row>
-    <row r="35" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="3" t="s">
         <v>2</v>
@@ -2504,7 +2504,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>19</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>20</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>21</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>22</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>23</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>24</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>25</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>26</v>
       </c>
@@ -2952,7 +2952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>27</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>28</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>29</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>30</v>
       </c>
@@ -3176,7 +3176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>31</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>32</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>33</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>34</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>35</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>36</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>37</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>38</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>39</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>40</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>41</v>
       </c>
@@ -3792,7 +3792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>42</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>43</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
         <v>44</v>
       </c>
@@ -3960,7 +3960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>45</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
         <v>46</v>
       </c>
@@ -4072,7 +4072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>47</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
         <v>49</v>
       </c>
@@ -4150,7 +4150,7 @@
       <c r="Q65" s="8"/>
       <c r="R65" s="8"/>
     </row>
-    <row r="66" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="3" t="s">
         <v>2</v>
@@ -4204,7 +4204,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>19</v>
       </c>
@@ -4260,7 +4260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>20</v>
       </c>
@@ -4316,7 +4316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>21</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>22</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>23</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>24</v>
       </c>
@@ -4540,7 +4540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>25</v>
       </c>
@@ -4596,7 +4596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>26</v>
       </c>
@@ -4652,7 +4652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>27</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>28</v>
       </c>
@@ -4764,7 +4764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>29</v>
       </c>
@@ -4820,7 +4820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>30</v>
       </c>
@@ -4876,7 +4876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>31</v>
       </c>
@@ -4932,7 +4932,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>32</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>33</v>
       </c>
@@ -5044,7 +5044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>34</v>
       </c>
@@ -5100,7 +5100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>35</v>
       </c>
@@ -5156,7 +5156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>36</v>
       </c>
@@ -5212,7 +5212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>37</v>
       </c>
@@ -5268,7 +5268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>38</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>39</v>
       </c>
@@ -5380,7 +5380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>40</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>41</v>
       </c>
@@ -5492,7 +5492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>42</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>43</v>
       </c>
@@ -5604,7 +5604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>44</v>
       </c>
@@ -5660,7 +5660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>45</v>
       </c>
@@ -5716,7 +5716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>46</v>
       </c>
@@ -5772,7 +5772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>47</v>
       </c>
@@ -5828,7 +5828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
         <v>50</v>
       </c>
@@ -5850,7 +5850,7 @@
       <c r="Q96" s="8"/>
       <c r="R96" s="8"/>
     </row>
-    <row r="97" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="3" t="s">
         <v>2</v>
@@ -5904,7 +5904,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
         <v>19</v>
       </c>
@@ -5960,7 +5960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
         <v>20</v>
       </c>
@@ -6016,7 +6016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
         <v>21</v>
       </c>
@@ -6072,7 +6072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
         <v>22</v>
       </c>
@@ -6128,7 +6128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
         <v>23</v>
       </c>
@@ -6184,7 +6184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
         <v>24</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
         <v>25</v>
       </c>
@@ -6296,7 +6296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
         <v>26</v>
       </c>
@@ -6352,7 +6352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
         <v>27</v>
       </c>
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>28</v>
       </c>
@@ -6464,7 +6464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>29</v>
       </c>
@@ -6520,7 +6520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>30</v>
       </c>
@@ -6576,7 +6576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
         <v>31</v>
       </c>
@@ -6632,7 +6632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
         <v>32</v>
       </c>
@@ -6688,7 +6688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
         <v>33</v>
       </c>
@@ -6744,7 +6744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
         <v>34</v>
       </c>
@@ -6800,7 +6800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>35</v>
       </c>
@@ -6856,7 +6856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
         <v>36</v>
       </c>
@@ -6912,7 +6912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
         <v>37</v>
       </c>
@@ -6968,7 +6968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
         <v>38</v>
       </c>
@@ -7024,7 +7024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
         <v>39</v>
       </c>
@@ -7080,7 +7080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
         <v>40</v>
       </c>
@@ -7136,7 +7136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
         <v>41</v>
       </c>
@@ -7192,7 +7192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
         <v>42</v>
       </c>
@@ -7248,7 +7248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
         <v>43</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
         <v>44</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
         <v>45</v>
       </c>
@@ -7416,7 +7416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
         <v>46</v>
       </c>
@@ -7472,7 +7472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
         <v>47</v>
       </c>
@@ -7528,7 +7528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
         <v>51</v>
       </c>
@@ -7562,7 +7562,7 @@
       <c r="AC127" s="8"/>
       <c r="AD127" s="8"/>
     </row>
-    <row r="128" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="3" t="s">
         <v>19</v>
@@ -7652,7 +7652,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="129" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
         <v>52</v>
       </c>
@@ -7744,7 +7744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
         <v>53</v>
       </c>
@@ -7836,7 +7836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
         <v>54</v>
       </c>
@@ -7857,7 +7857,7 @@
       <c r="P131" s="8"/>
       <c r="Q131" s="8"/>
     </row>
-    <row r="132" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>2</v>
       </c>
@@ -7910,7 +7910,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="133" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
         <v>55</v>
       </c>
@@ -7963,12 +7963,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="134" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="135" spans="1:30" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:30" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>2</v>
       </c>
@@ -8021,7 +8021,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="136" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>55</v>
       </c>
@@ -8074,12 +8074,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="137" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="138" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>0</v>
       </c>
@@ -8132,12 +8132,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="140" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A140" s="7">
         <v>0.5</v>
       </c>
@@ -8190,12 +8190,12 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="141" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="142" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>0</v>
       </c>
@@ -8248,12 +8248,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="144" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>0</v>
       </c>
@@ -8306,12 +8306,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>0</v>
       </c>
@@ -8364,7 +8364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>62</v>
       </c>
@@ -8379,5 +8379,6 @@
     <mergeCell ref="A127:AD127"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>